<commit_message>
docs: update project charter and business understanding
</commit_message>
<xml_diff>
--- a/01_Business_Understanding/Project_Charter.xlsx
+++ b/01_Business_Understanding/Project_Charter.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gplaneta-my.sharepoint.com/personal/umgz4a_psoplaneta_com/Documents/DATA/Analytics Projects/Product_Analytics/01_Business_Understanding/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="13" documentId="8_{2808834A-88FA-488B-A429-3D647F25CCEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BE8AC393-363B-47DA-AA9F-EDE9A3DF1B89}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="8_{2808834A-88FA-488B-A429-3D647F25CCEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{870972CE-0863-40BC-85C4-9AAE66D1A574}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="68">
   <si>
     <t>Fase ASUM-DM</t>
   </si>
@@ -273,12 +273,15 @@
   <si>
     <t>Proyecto dashboard de Inteligencia Competitiva de Precios y Demanda</t>
   </si>
+  <si>
+    <t>https://gplaneta-my.sharepoint.com/personal/umgz4a_psoplaneta_com/Documents/DATA/Analytics%20Projects/Product_Analytics/01_Business_Understanding</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -315,14 +318,6 @@
     <font>
       <u/>
       <sz val="11"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="9"/>
       <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -689,7 +684,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -729,9 +724,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="2" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -751,13 +743,13 @@
     </xf>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="6" xfId="3" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -879,6 +871,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="2" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -5000,7 +4995,7 @@
   <dimension ref="A1:J28"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.81640625" defaultRowHeight="10.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.81640625" style="18"/>
+    <col min="1" max="1" width="10.81640625" style="17"/>
     <col min="2" max="2" width="6.26953125" style="1" customWidth="1"/>
     <col min="3" max="4" width="10.81640625" style="1"/>
     <col min="5" max="5" width="15.26953125" style="1" customWidth="1"/>
@@ -5012,466 +5007,468 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="11" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="24" t="s">
         <v>51</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26"/>
-      <c r="I1" s="27"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+      <c r="I1" s="26"/>
     </row>
     <row r="2" spans="1:10" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="28" t="s">
+      <c r="A2" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="30" t="s">
+      <c r="B2" s="28"/>
+      <c r="C2" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
-      <c r="I2" s="31"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
+      <c r="I2" s="30"/>
     </row>
     <row r="3" spans="1:10" ht="11" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="25" t="s">
+      <c r="A3" s="24" t="s">
         <v>50</v>
       </c>
-      <c r="B3" s="26"/>
-      <c r="C3" s="26"/>
-      <c r="D3" s="26"/>
-      <c r="E3" s="26"/>
-      <c r="F3" s="26"/>
-      <c r="G3" s="26"/>
-      <c r="H3" s="26"/>
-      <c r="I3" s="27"/>
+      <c r="B3" s="25"/>
+      <c r="C3" s="25"/>
+      <c r="D3" s="25"/>
+      <c r="E3" s="25"/>
+      <c r="F3" s="25"/>
+      <c r="G3" s="25"/>
+      <c r="H3" s="25"/>
+      <c r="I3" s="26"/>
     </row>
     <row r="4" spans="1:10" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="43" t="s">
+      <c r="A4" s="42" t="s">
         <v>29</v>
       </c>
-      <c r="B4" s="44"/>
-      <c r="C4" s="39" t="s">
+      <c r="B4" s="43"/>
+      <c r="C4" s="38" t="s">
         <v>61</v>
       </c>
-      <c r="D4" s="39"/>
-      <c r="E4" s="39"/>
-      <c r="F4" s="39"/>
-      <c r="G4" s="39"/>
-      <c r="H4" s="39"/>
-      <c r="I4" s="40"/>
+      <c r="D4" s="38"/>
+      <c r="E4" s="38"/>
+      <c r="F4" s="38"/>
+      <c r="G4" s="38"/>
+      <c r="H4" s="38"/>
+      <c r="I4" s="39"/>
       <c r="J4" s="2"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="41" t="s">
+      <c r="A5" s="40" t="s">
         <v>30</v>
       </c>
-      <c r="B5" s="42"/>
-      <c r="C5" s="36" t="s">
+      <c r="B5" s="41"/>
+      <c r="C5" s="35" t="s">
         <v>62</v>
       </c>
-      <c r="D5" s="37"/>
-      <c r="E5" s="37"/>
-      <c r="F5" s="37"/>
-      <c r="G5" s="37"/>
-      <c r="H5" s="37"/>
-      <c r="I5" s="38"/>
+      <c r="D5" s="36"/>
+      <c r="E5" s="36"/>
+      <c r="F5" s="36"/>
+      <c r="G5" s="36"/>
+      <c r="H5" s="36"/>
+      <c r="I5" s="37"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" s="41"/>
-      <c r="B6" s="42"/>
-      <c r="C6" s="37"/>
-      <c r="D6" s="37"/>
-      <c r="E6" s="37"/>
-      <c r="F6" s="37"/>
-      <c r="G6" s="37"/>
-      <c r="H6" s="37"/>
-      <c r="I6" s="38"/>
+      <c r="A6" s="40"/>
+      <c r="B6" s="41"/>
+      <c r="C6" s="36"/>
+      <c r="D6" s="36"/>
+      <c r="E6" s="36"/>
+      <c r="F6" s="36"/>
+      <c r="G6" s="36"/>
+      <c r="H6" s="36"/>
+      <c r="I6" s="37"/>
     </row>
     <row r="7" spans="1:10" ht="86.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="41"/>
-      <c r="B7" s="42"/>
-      <c r="C7" s="37"/>
-      <c r="D7" s="37"/>
-      <c r="E7" s="37"/>
-      <c r="F7" s="37"/>
-      <c r="G7" s="37"/>
-      <c r="H7" s="37"/>
-      <c r="I7" s="38"/>
+      <c r="A7" s="40"/>
+      <c r="B7" s="41"/>
+      <c r="C7" s="36"/>
+      <c r="D7" s="36"/>
+      <c r="E7" s="36"/>
+      <c r="F7" s="36"/>
+      <c r="G7" s="36"/>
+      <c r="H7" s="36"/>
+      <c r="I7" s="37"/>
       <c r="J7" s="1" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="34.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="32" t="s">
+      <c r="A8" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="B8" s="33"/>
-      <c r="C8" s="34" t="s">
+      <c r="B8" s="32"/>
+      <c r="C8" s="33" t="s">
         <v>52</v>
       </c>
-      <c r="D8" s="34"/>
-      <c r="E8" s="34"/>
-      <c r="F8" s="34"/>
-      <c r="G8" s="34"/>
-      <c r="H8" s="34"/>
-      <c r="I8" s="35"/>
+      <c r="D8" s="33"/>
+      <c r="E8" s="33"/>
+      <c r="F8" s="33"/>
+      <c r="G8" s="33"/>
+      <c r="H8" s="33"/>
+      <c r="I8" s="34"/>
     </row>
     <row r="9" spans="1:10" ht="11" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="25" t="s">
+      <c r="A9" s="24" t="s">
         <v>33</v>
       </c>
-      <c r="B9" s="26"/>
-      <c r="C9" s="26"/>
-      <c r="D9" s="26"/>
-      <c r="E9" s="26"/>
-      <c r="F9" s="26"/>
-      <c r="G9" s="26"/>
-      <c r="H9" s="26"/>
-      <c r="I9" s="27"/>
+      <c r="B9" s="25"/>
+      <c r="C9" s="25"/>
+      <c r="D9" s="25"/>
+      <c r="E9" s="25"/>
+      <c r="F9" s="25"/>
+      <c r="G9" s="25"/>
+      <c r="H9" s="25"/>
+      <c r="I9" s="26"/>
     </row>
     <row r="10" spans="1:10" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="47" t="s">
+      <c r="A10" s="46" t="s">
         <v>34</v>
       </c>
-      <c r="B10" s="48"/>
-      <c r="C10" s="49" t="s">
+      <c r="B10" s="47"/>
+      <c r="C10" s="48" t="s">
         <v>65</v>
       </c>
-      <c r="D10" s="49"/>
-      <c r="E10" s="49"/>
-      <c r="F10" s="49"/>
-      <c r="G10" s="49"/>
-      <c r="H10" s="49"/>
-      <c r="I10" s="50"/>
+      <c r="D10" s="48"/>
+      <c r="E10" s="48"/>
+      <c r="F10" s="48"/>
+      <c r="G10" s="48"/>
+      <c r="H10" s="48"/>
+      <c r="I10" s="49"/>
     </row>
     <row r="11" spans="1:10" ht="26.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="52" t="s">
+      <c r="A11" s="51" t="s">
         <v>35</v>
       </c>
-      <c r="B11" s="53"/>
-      <c r="C11" s="51" t="s">
+      <c r="B11" s="52"/>
+      <c r="C11" s="50" t="s">
         <v>36</v>
       </c>
-      <c r="D11" s="51"/>
-      <c r="E11" s="51"/>
-      <c r="F11" s="51"/>
-      <c r="G11" s="51"/>
-      <c r="H11" s="21" t="s">
+      <c r="D11" s="50"/>
+      <c r="E11" s="50"/>
+      <c r="F11" s="50"/>
+      <c r="G11" s="50"/>
+      <c r="H11" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="I11" s="22" t="s">
+      <c r="I11" s="21" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="52"/>
-      <c r="B12" s="53"/>
-      <c r="C12" s="45" t="s">
+      <c r="A12" s="51"/>
+      <c r="B12" s="52"/>
+      <c r="C12" s="44" t="s">
         <v>63</v>
       </c>
-      <c r="D12" s="45"/>
-      <c r="E12" s="45"/>
-      <c r="F12" s="45"/>
-      <c r="G12" s="45"/>
-      <c r="H12" s="23">
+      <c r="D12" s="44"/>
+      <c r="E12" s="44"/>
+      <c r="F12" s="44"/>
+      <c r="G12" s="44"/>
+      <c r="H12" s="22">
         <v>0</v>
       </c>
-      <c r="I12" s="24">
+      <c r="I12" s="23">
         <v>0.95</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="52"/>
-      <c r="B13" s="53"/>
-      <c r="C13" s="45" t="s">
+      <c r="A13" s="51"/>
+      <c r="B13" s="52"/>
+      <c r="C13" s="44" t="s">
         <v>53</v>
       </c>
-      <c r="D13" s="45"/>
-      <c r="E13" s="45"/>
-      <c r="F13" s="45"/>
-      <c r="G13" s="45"/>
-      <c r="H13" s="23">
+      <c r="D13" s="44"/>
+      <c r="E13" s="44"/>
+      <c r="F13" s="44"/>
+      <c r="G13" s="44"/>
+      <c r="H13" s="22">
         <v>0</v>
       </c>
-      <c r="I13" s="24">
+      <c r="I13" s="23">
         <v>0.95</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="52"/>
-      <c r="B14" s="53"/>
-      <c r="C14" s="45" t="s">
+      <c r="A14" s="51"/>
+      <c r="B14" s="52"/>
+      <c r="C14" s="44" t="s">
         <v>54</v>
       </c>
-      <c r="D14" s="45"/>
-      <c r="E14" s="45"/>
-      <c r="F14" s="45"/>
-      <c r="G14" s="45"/>
-      <c r="H14" s="16">
+      <c r="D14" s="44"/>
+      <c r="E14" s="44"/>
+      <c r="F14" s="44"/>
+      <c r="G14" s="44"/>
+      <c r="H14" s="15">
         <v>0</v>
       </c>
-      <c r="I14" s="17" t="s">
+      <c r="I14" s="16" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="52"/>
-      <c r="B15" s="53"/>
-      <c r="C15" s="45" t="s">
+      <c r="A15" s="51"/>
+      <c r="B15" s="52"/>
+      <c r="C15" s="44" t="s">
         <v>56</v>
       </c>
-      <c r="D15" s="45"/>
-      <c r="E15" s="45"/>
-      <c r="F15" s="45"/>
-      <c r="G15" s="45"/>
-      <c r="H15" s="16">
+      <c r="D15" s="44"/>
+      <c r="E15" s="44"/>
+      <c r="F15" s="44"/>
+      <c r="G15" s="44"/>
+      <c r="H15" s="15">
         <v>0</v>
       </c>
-      <c r="I15" s="24">
+      <c r="I15" s="23">
         <v>0.95</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="41" t="s">
+      <c r="A16" s="40" t="s">
         <v>39</v>
       </c>
-      <c r="B16" s="42"/>
-      <c r="C16" s="45" t="s">
+      <c r="B16" s="41"/>
+      <c r="C16" s="44" t="s">
         <v>64</v>
       </c>
-      <c r="D16" s="45"/>
-      <c r="E16" s="45"/>
-      <c r="F16" s="42" t="s">
+      <c r="D16" s="44"/>
+      <c r="E16" s="44"/>
+      <c r="F16" s="41" t="s">
         <v>40</v>
       </c>
-      <c r="G16" s="42"/>
-      <c r="H16" s="45" t="s">
+      <c r="G16" s="41"/>
+      <c r="H16" s="44" t="s">
         <v>57</v>
       </c>
-      <c r="I16" s="46"/>
+      <c r="I16" s="45"/>
     </row>
     <row r="17" spans="1:9" ht="179.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="41"/>
-      <c r="B17" s="42"/>
-      <c r="C17" s="45"/>
-      <c r="D17" s="45"/>
-      <c r="E17" s="45"/>
-      <c r="F17" s="42"/>
-      <c r="G17" s="42"/>
-      <c r="H17" s="45"/>
-      <c r="I17" s="46"/>
+      <c r="A17" s="40"/>
+      <c r="B17" s="41"/>
+      <c r="C17" s="44"/>
+      <c r="D17" s="44"/>
+      <c r="E17" s="44"/>
+      <c r="F17" s="41"/>
+      <c r="G17" s="41"/>
+      <c r="H17" s="44"/>
+      <c r="I17" s="45"/>
     </row>
     <row r="18" spans="1:9" ht="30.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="41" t="s">
+      <c r="A18" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="B18" s="42"/>
-      <c r="C18" s="45" t="s">
+      <c r="B18" s="41"/>
+      <c r="C18" s="44" t="s">
         <v>58</v>
       </c>
-      <c r="D18" s="45"/>
-      <c r="E18" s="45"/>
-      <c r="F18" s="45"/>
-      <c r="G18" s="45"/>
-      <c r="H18" s="45"/>
-      <c r="I18" s="46"/>
+      <c r="D18" s="44"/>
+      <c r="E18" s="44"/>
+      <c r="F18" s="44"/>
+      <c r="G18" s="44"/>
+      <c r="H18" s="44"/>
+      <c r="I18" s="45"/>
     </row>
     <row r="19" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="41" t="s">
+      <c r="A19" s="40" t="s">
         <v>42</v>
       </c>
-      <c r="B19" s="42"/>
-      <c r="C19" s="62" t="s">
+      <c r="B19" s="41"/>
+      <c r="C19" s="61" t="s">
         <v>36</v>
       </c>
-      <c r="D19" s="62"/>
-      <c r="E19" s="62"/>
-      <c r="F19" s="62"/>
-      <c r="G19" s="62" t="s">
+      <c r="D19" s="61"/>
+      <c r="E19" s="61"/>
+      <c r="F19" s="61"/>
+      <c r="G19" s="61" t="s">
         <v>43</v>
       </c>
-      <c r="H19" s="62"/>
-      <c r="I19" s="63"/>
+      <c r="H19" s="61"/>
+      <c r="I19" s="62"/>
     </row>
     <row r="20" spans="1:9" ht="11" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="60"/>
-      <c r="B20" s="61"/>
-      <c r="C20" s="54" t="s">
+      <c r="A20" s="59"/>
+      <c r="B20" s="60"/>
+      <c r="C20" s="53" t="s">
         <v>44</v>
       </c>
-      <c r="D20" s="54"/>
-      <c r="E20" s="54"/>
-      <c r="F20" s="54"/>
-      <c r="G20" s="54" t="s">
+      <c r="D20" s="53"/>
+      <c r="E20" s="53"/>
+      <c r="F20" s="53"/>
+      <c r="G20" s="53" t="s">
         <v>45</v>
       </c>
-      <c r="H20" s="54"/>
-      <c r="I20" s="55"/>
+      <c r="H20" s="53"/>
+      <c r="I20" s="54"/>
     </row>
     <row r="21" spans="1:9" ht="11" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="25" t="s">
+      <c r="A21" s="24" t="s">
         <v>46</v>
       </c>
-      <c r="B21" s="26"/>
-      <c r="C21" s="26"/>
-      <c r="D21" s="26"/>
-      <c r="E21" s="26"/>
-      <c r="F21" s="26"/>
-      <c r="G21" s="26"/>
-      <c r="H21" s="26"/>
-      <c r="I21" s="27"/>
+      <c r="B21" s="25"/>
+      <c r="C21" s="25"/>
+      <c r="D21" s="25"/>
+      <c r="E21" s="25"/>
+      <c r="F21" s="25"/>
+      <c r="G21" s="25"/>
+      <c r="H21" s="25"/>
+      <c r="I21" s="26"/>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22" s="58" t="s">
+      <c r="A22" s="57" t="s">
         <v>47</v>
       </c>
-      <c r="B22" s="59"/>
-      <c r="C22" s="19" t="s">
+      <c r="B22" s="58"/>
+      <c r="C22" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="D22" s="59" t="s">
+      <c r="D22" s="58" t="s">
         <v>2</v>
       </c>
-      <c r="E22" s="59"/>
-      <c r="F22" s="59" t="s">
+      <c r="E22" s="58"/>
+      <c r="F22" s="58" t="s">
         <v>3</v>
       </c>
-      <c r="G22" s="59"/>
-      <c r="H22" s="19" t="s">
+      <c r="G22" s="58"/>
+      <c r="H22" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="I22" s="20" t="s">
+      <c r="I22" s="19" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="23" spans="1:9" s="11" customFormat="1" ht="49.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="56" t="s">
+      <c r="A23" s="55" t="s">
         <v>4</v>
       </c>
-      <c r="B23" s="57"/>
+      <c r="B23" s="56"/>
       <c r="C23" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="D23" s="64" t="s">
+      <c r="D23" s="63" t="s">
         <v>6</v>
       </c>
-      <c r="E23" s="64"/>
-      <c r="F23" s="64" t="s">
+      <c r="E23" s="63"/>
+      <c r="F23" s="63" t="s">
         <v>7</v>
       </c>
-      <c r="G23" s="64"/>
-      <c r="H23" s="15"/>
+      <c r="G23" s="63"/>
+      <c r="H23" s="67" t="s">
+        <v>67</v>
+      </c>
       <c r="I23" s="10" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="24" spans="1:9" s="11" customFormat="1" ht="64" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="56" t="s">
+      <c r="A24" s="55" t="s">
         <v>8</v>
       </c>
-      <c r="B24" s="57"/>
+      <c r="B24" s="56"/>
       <c r="C24" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="D24" s="64" t="s">
+      <c r="D24" s="63" t="s">
         <v>10</v>
       </c>
-      <c r="E24" s="64"/>
-      <c r="F24" s="64" t="s">
+      <c r="E24" s="63"/>
+      <c r="F24" s="63" t="s">
         <v>11</v>
       </c>
-      <c r="G24" s="64"/>
+      <c r="G24" s="63"/>
       <c r="H24" s="9"/>
       <c r="I24" s="10" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="25" spans="1:9" s="11" customFormat="1" ht="52.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="56" t="s">
+      <c r="A25" s="55" t="s">
         <v>12</v>
       </c>
-      <c r="B25" s="57"/>
+      <c r="B25" s="56"/>
       <c r="C25" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="D25" s="64" t="s">
+      <c r="D25" s="63" t="s">
         <v>14</v>
       </c>
-      <c r="E25" s="64"/>
-      <c r="F25" s="64" t="s">
+      <c r="E25" s="63"/>
+      <c r="F25" s="63" t="s">
         <v>15</v>
       </c>
-      <c r="G25" s="64"/>
+      <c r="G25" s="63"/>
       <c r="H25" s="9"/>
       <c r="I25" s="10" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="26" spans="1:9" s="11" customFormat="1" ht="52.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="56" t="s">
+      <c r="A26" s="55" t="s">
         <v>16</v>
       </c>
-      <c r="B26" s="57"/>
+      <c r="B26" s="56"/>
       <c r="C26" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="D26" s="64" t="s">
+      <c r="D26" s="63" t="s">
         <v>18</v>
       </c>
-      <c r="E26" s="64"/>
-      <c r="F26" s="64" t="s">
+      <c r="E26" s="63"/>
+      <c r="F26" s="63" t="s">
         <v>19</v>
       </c>
-      <c r="G26" s="64"/>
+      <c r="G26" s="63"/>
       <c r="H26" s="9"/>
       <c r="I26" s="10" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="27" spans="1:9" s="11" customFormat="1" ht="52.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="56" t="s">
+      <c r="A27" s="55" t="s">
         <v>20</v>
       </c>
-      <c r="B27" s="57"/>
+      <c r="B27" s="56"/>
       <c r="C27" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="D27" s="64" t="s">
+      <c r="D27" s="63" t="s">
         <v>22</v>
       </c>
-      <c r="E27" s="64"/>
-      <c r="F27" s="64" t="s">
+      <c r="E27" s="63"/>
+      <c r="F27" s="63" t="s">
         <v>23</v>
       </c>
-      <c r="G27" s="64"/>
+      <c r="G27" s="63"/>
       <c r="H27" s="9"/>
       <c r="I27" s="10" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="28" spans="1:9" s="11" customFormat="1" ht="44.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A28" s="66" t="s">
+      <c r="A28" s="65" t="s">
         <v>24</v>
       </c>
-      <c r="B28" s="67"/>
+      <c r="B28" s="66"/>
       <c r="C28" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="D28" s="65" t="s">
+      <c r="D28" s="64" t="s">
         <v>26</v>
       </c>
-      <c r="E28" s="65"/>
-      <c r="F28" s="65" t="s">
+      <c r="E28" s="64"/>
+      <c r="F28" s="64" t="s">
         <v>27</v>
       </c>
-      <c r="G28" s="65"/>
+      <c r="G28" s="64"/>
       <c r="H28" s="13"/>
       <c r="I28" s="14" t="s">
         <v>59</v>
@@ -5532,8 +5529,11 @@
     <mergeCell ref="A5:B7"/>
     <mergeCell ref="A4:B4"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="H23" r:id="rId1" xr:uid="{4A9A01C2-595E-46B3-82AB-AA30192D9F42}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
docs: update project charter 2 and business understanding
</commit_message>
<xml_diff>
--- a/01_Business_Understanding/Project_Charter.xlsx
+++ b/01_Business_Understanding/Project_Charter.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gplaneta-my.sharepoint.com/personal/umgz4a_psoplaneta_com/Documents/DATA/Analytics Projects/Product_Analytics/01_Business_Understanding/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="8_{2808834A-88FA-488B-A429-3D647F25CCEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{870972CE-0863-40BC-85C4-9AAE66D1A574}"/>
+  <xr:revisionPtr revIDLastSave="18" documentId="8_{2808834A-88FA-488B-A429-3D647F25CCEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{014E6DFA-6E41-4109-B66E-2D0B085214A0}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -274,14 +274,14 @@
     <t>Proyecto dashboard de Inteligencia Competitiva de Precios y Demanda</t>
   </si>
   <si>
-    <t>https://gplaneta-my.sharepoint.com/personal/umgz4a_psoplaneta_com/Documents/DATA/Analytics%20Projects/Product_Analytics/01_Business_Understanding</t>
+    <t>01_Business_Understanding</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -335,6 +335,14 @@
       <color theme="1"/>
       <name val="Aptos"/>
     </font>
+    <font>
+      <u/>
+      <sz val="8"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -872,7 +880,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="2" quotePrefix="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="2" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>

</xml_diff>